<commit_message>
updated excel sheet for specific
</commit_message>
<xml_diff>
--- a/pilots_and_power/rating_data/explaining_alteration_differences.xlsx
+++ b/pilots_and_power/rating_data/explaining_alteration_differences.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="38">
   <si>
     <t xml:space="preserve">Timestamp_sum</t>
   </si>
@@ -56,9 +56,6 @@
   </si>
   <si>
     <t xml:space="preserve">Legal fees, vicar? Reverend, 63, who was jailed for Just Stop Oil protest outside fuel terminal - breaking a court injunction - launches fundraiser to pay £2,000 bill</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arguably not specific, but summary seemed specific</t>
   </si>
   <si>
     <t xml:space="preserve">Blockade, Protesters physically attached to or on top of something, Breaching a legal injunction</t>
@@ -290,120 +287,120 @@
         <v>11</v>
       </c>
       <c r="E2" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="G2" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="H2" s="0" t="s">
         <v>14</v>
-      </c>
-      <c r="H2" s="0" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B3" s="0" t="s">
         <v>9</v>
       </c>
       <c r="C3" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="E3" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="F3" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="G3" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="0" t="s">
         <v>20</v>
-      </c>
-      <c r="G3" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" s="0" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B4" s="0" t="s">
         <v>9</v>
       </c>
       <c r="C4" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="E4" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="F4" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="0" t="s">
         <v>25</v>
-      </c>
-      <c r="F4" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="0" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B5" s="0" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="E5" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="F5" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="G5" s="0" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="G5" s="0" t="s">
+      <c r="H5" s="0" t="s">
         <v>31</v>
-      </c>
-      <c r="H5" s="0" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B6" s="0" t="s">
         <v>9</v>
       </c>
       <c r="C6" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="0" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="E6" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="0" t="s">
         <v>35</v>
       </c>
-      <c r="E6" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" s="0" t="s">
+      <c r="G6" s="0" t="s">
         <v>36</v>
       </c>
-      <c r="G6" s="0" t="s">
+      <c r="H6" s="0" t="s">
         <v>37</v>
-      </c>
-      <c r="H6" s="0" t="s">
-        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>